<commit_message>
bonus plants and zombies added.
</commit_message>
<xml_diff>
--- a/ap project documents/AP_project_2026_one_team_tracker.xlsx
+++ b/ap project documents/AP_project_2026_one_team_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arian\Desktop\uni\AP\Project\Plants-vs-Zombies-2\ap project documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5747C909-1957-4C91-8EFE-EE2AE2065727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E8464E5-9CFE-42EE-8D32-2D1E2B7BFD2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="B14" s="37">
         <f>_logic_p2!II5</f>
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="C14" s="31">
         <f>_logic_p2!II4</f>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="D14" s="34">
         <f t="shared" si="0"/>
-        <v>2.3952095808383235E-2</v>
+        <v>0.12574850299401197</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="55"/>
@@ -10432,7 +10432,7 @@
       <c r="F8" s="61"/>
       <c r="G8" s="61" t="str">
         <f>_logic_p2!II5&amp;" / "&amp;_logic_p2!II4</f>
-        <v>20 / 835</v>
+        <v>105 / 835</v>
       </c>
       <c r="H8" s="61"/>
     </row>
@@ -17505,20 +17505,20 @@
         <v>55</v>
       </c>
       <c r="E206" s="17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F206" s="20"/>
       <c r="G206" s="23">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="H206" s="14">
         <f t="shared" si="10"/>
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="I206" s="10" t="str">
         <f t="shared" si="11"/>
-        <v>Do: گیاهان امتیازی</v>
+        <v>Done</v>
       </c>
       <c r="J206" s="39" t="s">
         <v>156</v>
@@ -17541,20 +17541,20 @@
         <v>30</v>
       </c>
       <c r="E207" s="17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F207" s="20"/>
       <c r="G207" s="23">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H207" s="14">
         <f t="shared" si="10"/>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I207" s="10" t="str">
         <f t="shared" si="11"/>
-        <v>Do: زامبی‌های امتیازی</v>
+        <v>Done</v>
       </c>
       <c r="J207" s="39" t="s">
         <v>156</v>
@@ -23959,11 +23959,11 @@
       </c>
       <c r="GO5" s="28">
         <f>'Phase 2'!G206</f>
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="GP5" s="28">
         <f>'Phase 2'!G207</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="GQ5" s="28">
         <f>'Phase 2'!G208</f>
@@ -24131,7 +24131,7 @@
       </c>
       <c r="II5" s="28">
         <f>MIN(SUM(GO5:IA5,MAX(IG5+IF5-IF4,0)/3),II4)</f>
-        <v>20</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>